<commit_message>
config: adiciona traducoes i18n para pt-BR e padroniza coluna para nome
</commit_message>
<xml_diff>
--- a/spec/fixtures/files/mixed_import.xlsx
+++ b/spec/fixtures/files/mixed_import.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr date1904="false"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" r:id="rId1"/>
+    <sheet sheetId="1" name="Basic Worksheet" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -342,19 +342,19 @@
       </c>
       <c r="B1" s="0" t="inlineStr">
         <is>
-          <t>full_name</t>
+          <t>nome</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>heidi@example.com</t>
+          <t>dave@example.com</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>Heidi Example</t>
+          <t>Dave Example</t>
         </is>
       </c>
     </row>
@@ -397,12 +397,12 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>ivan@example.com</t>
+          <t>erin@example.com</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>Ivan Example</t>
+          <t>Erin Example</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: cover the headerless spreadsheet import toggle
Reorders every CSV/XLSX fixture to name-first/email-second (the new positional
contract) and adds coverage for both has_header states: the header row is never
used to map columns (even when its labels don't say nome/email), and a file
without a header is read from row 1 onward.
</commit_message>
<xml_diff>
--- a/spec/fixtures/files/mixed_import.xlsx
+++ b/spec/fixtures/files/mixed_import.xlsx
@@ -323,7 +323,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+<worksheet space="preserve">
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
@@ -337,72 +337,72 @@
     <row r="1">
       <c r="A1" s="0" t="inlineStr">
         <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
           <t>email</t>
-        </is>
-      </c>
-      <c r="B1" s="0" t="inlineStr">
-        <is>
-          <t>nome</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
+          <t>Dave Example</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
           <t>dave@example.com</t>
-        </is>
-      </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t>Dave Example</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
+          <t>Missing Email</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
           <t/>
-        </is>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>Missing Email</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
+          <t>Bad Email Format</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
           <t>not-an-email</t>
-        </is>
-      </c>
-      <c r="B4" s="0" t="inlineStr">
-        <is>
-          <t>Bad Email Format</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
+          <t>Duplicate Email</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
           <t>existing@example.com</t>
-        </is>
-      </c>
-      <c r="B5" s="0" t="inlineStr">
-        <is>
-          <t>Duplicate Email</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
+          <t>Erin Example</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
           <t>erin@example.com</t>
-        </is>
-      </c>
-      <c r="B6" s="0" t="inlineStr">
-        <is>
-          <t>Erin Example</t>
         </is>
       </c>
     </row>

</xml_diff>